<commit_message>
new file:   data/FRS_cleaned/FRS/Dec/Fmn A Dec/Dec 2025-A.xlsx
</commit_message>
<xml_diff>
--- a/data/FRS_cleaned/Nov/Fmn G Nov/Nov 2025-G.xlsx
+++ b/data/FRS_cleaned/Nov/Fmn G Nov/Nov 2025-G.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B84FE1B2-FD2B-4C14-B159-1E416B891CEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{27206D68-33BE-482D-802F-57DE02E6DC52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="A Vehicle" sheetId="20" r:id="rId1"/>
@@ -5009,41 +5009,44 @@
       <alignment vertical="top" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -5113,12 +5116,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -5208,38 +5205,41 @@
     <xf numFmtId="2" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="10">
@@ -5601,80 +5601,80 @@
       <c r="U2" s="92"/>
     </row>
     <row r="3" spans="1:21" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A3" s="374" t="s">
+      <c r="A3" s="375" t="s">
         <v>392</v>
       </c>
-      <c r="B3" s="374"/>
-      <c r="C3" s="374"/>
-      <c r="D3" s="374"/>
-      <c r="E3" s="374"/>
-      <c r="F3" s="374"/>
-      <c r="G3" s="374"/>
-      <c r="H3" s="374"/>
-      <c r="I3" s="374"/>
-      <c r="J3" s="374"/>
-      <c r="K3" s="374"/>
-      <c r="L3" s="374"/>
-      <c r="M3" s="374"/>
-      <c r="N3" s="374"/>
-      <c r="O3" s="374"/>
-      <c r="P3" s="374"/>
-      <c r="Q3" s="374"/>
-      <c r="R3" s="374"/>
-      <c r="S3" s="374"/>
-      <c r="T3" s="374"/>
-      <c r="U3" s="374"/>
+      <c r="B3" s="375"/>
+      <c r="C3" s="375"/>
+      <c r="D3" s="375"/>
+      <c r="E3" s="375"/>
+      <c r="F3" s="375"/>
+      <c r="G3" s="375"/>
+      <c r="H3" s="375"/>
+      <c r="I3" s="375"/>
+      <c r="J3" s="375"/>
+      <c r="K3" s="375"/>
+      <c r="L3" s="375"/>
+      <c r="M3" s="375"/>
+      <c r="N3" s="375"/>
+      <c r="O3" s="375"/>
+      <c r="P3" s="375"/>
+      <c r="Q3" s="375"/>
+      <c r="R3" s="375"/>
+      <c r="S3" s="375"/>
+      <c r="T3" s="375"/>
+      <c r="U3" s="375"/>
     </row>
     <row r="4" spans="1:21" s="19" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A4" s="375" t="s">
+      <c r="A4" s="376" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="373" t="s">
+      <c r="B4" s="374" t="s">
         <v>14</v>
       </c>
       <c r="C4" s="39"/>
-      <c r="D4" s="375" t="s">
+      <c r="D4" s="376" t="s">
         <v>19</v>
       </c>
-      <c r="E4" s="375"/>
-      <c r="F4" s="375" t="s">
+      <c r="E4" s="376"/>
+      <c r="F4" s="376" t="s">
         <v>33</v>
       </c>
-      <c r="G4" s="375"/>
-      <c r="H4" s="375"/>
-      <c r="I4" s="375"/>
-      <c r="J4" s="375"/>
-      <c r="K4" s="375"/>
-      <c r="L4" s="375"/>
-      <c r="M4" s="375"/>
-      <c r="N4" s="373" t="s">
+      <c r="G4" s="376"/>
+      <c r="H4" s="376"/>
+      <c r="I4" s="376"/>
+      <c r="J4" s="376"/>
+      <c r="K4" s="376"/>
+      <c r="L4" s="376"/>
+      <c r="M4" s="376"/>
+      <c r="N4" s="374" t="s">
         <v>20</v>
       </c>
-      <c r="O4" s="373" t="s">
+      <c r="O4" s="374" t="s">
         <v>34</v>
       </c>
-      <c r="P4" s="375" t="s">
+      <c r="P4" s="376" t="s">
         <v>35</v>
       </c>
-      <c r="Q4" s="373" t="s">
+      <c r="Q4" s="374" t="s">
         <v>23</v>
       </c>
-      <c r="R4" s="373" t="s">
+      <c r="R4" s="374" t="s">
         <v>24</v>
       </c>
-      <c r="S4" s="373" t="s">
+      <c r="S4" s="374" t="s">
         <v>25</v>
       </c>
-      <c r="T4" s="373" t="s">
+      <c r="T4" s="374" t="s">
         <v>26</v>
       </c>
-      <c r="U4" s="373" t="s">
+      <c r="U4" s="374" t="s">
         <v>156</v>
       </c>
     </row>
     <row r="5" spans="1:21" s="19" customFormat="1" ht="41.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="375"/>
-      <c r="B5" s="373"/>
+      <c r="A5" s="376"/>
+      <c r="B5" s="374"/>
       <c r="C5" s="39" t="s">
         <v>612</v>
       </c>
@@ -5708,14 +5708,14 @@
       <c r="M5" s="40" t="s">
         <v>30</v>
       </c>
-      <c r="N5" s="373"/>
-      <c r="O5" s="373"/>
-      <c r="P5" s="375"/>
-      <c r="Q5" s="373"/>
-      <c r="R5" s="373"/>
-      <c r="S5" s="373"/>
-      <c r="T5" s="373"/>
-      <c r="U5" s="373"/>
+      <c r="N5" s="374"/>
+      <c r="O5" s="374"/>
+      <c r="P5" s="376"/>
+      <c r="Q5" s="374"/>
+      <c r="R5" s="374"/>
+      <c r="S5" s="374"/>
+      <c r="T5" s="374"/>
+      <c r="U5" s="374"/>
     </row>
     <row r="6" spans="1:21" s="19" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A6" s="40" t="s">
@@ -5781,10 +5781,10 @@
       </c>
     </row>
     <row r="7" spans="1:21" s="19" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="372" t="s">
+      <c r="A7" s="373" t="s">
         <v>153</v>
       </c>
-      <c r="B7" s="372"/>
+      <c r="B7" s="373"/>
       <c r="C7" s="46"/>
       <c r="D7" s="40"/>
       <c r="E7" s="40"/>
@@ -6925,57 +6925,57 @@
       <c r="G1" s="224"/>
       <c r="H1" s="224"/>
       <c r="I1" s="224"/>
-      <c r="J1" s="425" t="s">
+      <c r="J1" s="360" t="s">
         <v>1100</v>
       </c>
-      <c r="K1" s="425"/>
-      <c r="L1" s="425"/>
+      <c r="K1" s="360"/>
+      <c r="L1" s="360"/>
     </row>
     <row r="2" spans="1:12" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="426" t="s">
+      <c r="A2" s="361" t="s">
         <v>1101</v>
       </c>
-      <c r="B2" s="426"/>
-      <c r="C2" s="426"/>
-      <c r="D2" s="426"/>
-      <c r="E2" s="426"/>
-      <c r="F2" s="426"/>
-      <c r="G2" s="426"/>
-      <c r="H2" s="426"/>
-      <c r="I2" s="426"/>
-      <c r="J2" s="426"/>
+      <c r="B2" s="361"/>
+      <c r="C2" s="361"/>
+      <c r="D2" s="361"/>
+      <c r="E2" s="361"/>
+      <c r="F2" s="361"/>
+      <c r="G2" s="361"/>
+      <c r="H2" s="361"/>
+      <c r="I2" s="361"/>
+      <c r="J2" s="361"/>
     </row>
     <row r="3" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="395" t="s">
+      <c r="A3" s="371" t="s">
         <v>1102</v>
       </c>
-      <c r="B3" s="395" t="s">
+      <c r="B3" s="371" t="s">
         <v>1103</v>
       </c>
-      <c r="C3" s="427" t="s">
+      <c r="C3" s="362" t="s">
         <v>1112</v>
       </c>
-      <c r="D3" s="428"/>
-      <c r="E3" s="427" t="s">
+      <c r="D3" s="363"/>
+      <c r="E3" s="362" t="s">
         <v>1113</v>
       </c>
-      <c r="F3" s="429"/>
-      <c r="G3" s="429"/>
-      <c r="H3" s="429"/>
-      <c r="I3" s="428"/>
-      <c r="J3" s="430" t="s">
+      <c r="F3" s="364"/>
+      <c r="G3" s="364"/>
+      <c r="H3" s="364"/>
+      <c r="I3" s="363"/>
+      <c r="J3" s="365" t="s">
         <v>1113</v>
       </c>
-      <c r="K3" s="432" t="s">
+      <c r="K3" s="367" t="s">
         <v>1118</v>
       </c>
-      <c r="L3" s="434" t="s">
+      <c r="L3" s="369" t="s">
         <v>1104</v>
       </c>
     </row>
     <row r="4" spans="1:12" ht="15.6" x14ac:dyDescent="0.25">
-      <c r="A4" s="396"/>
-      <c r="B4" s="396"/>
+      <c r="A4" s="372"/>
+      <c r="B4" s="372"/>
       <c r="C4" s="353" t="s">
         <v>1114</v>
       </c>
@@ -6997,9 +6997,9 @@
       <c r="I4" s="353" t="s">
         <v>1117</v>
       </c>
-      <c r="J4" s="431"/>
-      <c r="K4" s="433"/>
-      <c r="L4" s="435"/>
+      <c r="J4" s="366"/>
+      <c r="K4" s="368"/>
+      <c r="L4" s="370"/>
     </row>
     <row r="5" spans="1:12" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="72">
@@ -7217,44 +7217,44 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="376" t="s">
+      <c r="A1" s="377" t="s">
         <v>915</v>
       </c>
-      <c r="B1" s="377"/>
-      <c r="C1" s="377"/>
-      <c r="D1" s="378"/>
-      <c r="E1" s="377"/>
-      <c r="F1" s="377"/>
-      <c r="G1" s="377"/>
-      <c r="H1" s="377"/>
-      <c r="I1" s="377"/>
-      <c r="J1" s="377"/>
+      <c r="B1" s="378"/>
+      <c r="C1" s="378"/>
+      <c r="D1" s="379"/>
+      <c r="E1" s="378"/>
+      <c r="F1" s="378"/>
+      <c r="G1" s="378"/>
+      <c r="H1" s="378"/>
+      <c r="I1" s="378"/>
+      <c r="J1" s="378"/>
     </row>
     <row r="2" spans="1:38" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="377"/>
-      <c r="B2" s="377"/>
-      <c r="C2" s="377"/>
-      <c r="D2" s="378"/>
-      <c r="E2" s="377"/>
-      <c r="F2" s="377"/>
-      <c r="G2" s="377"/>
-      <c r="H2" s="377"/>
-      <c r="I2" s="377"/>
-      <c r="J2" s="377"/>
+      <c r="A2" s="378"/>
+      <c r="B2" s="378"/>
+      <c r="C2" s="378"/>
+      <c r="D2" s="379"/>
+      <c r="E2" s="378"/>
+      <c r="F2" s="378"/>
+      <c r="G2" s="378"/>
+      <c r="H2" s="378"/>
+      <c r="I2" s="378"/>
+      <c r="J2" s="378"/>
     </row>
     <row r="3" spans="1:38" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="377" t="s">
+      <c r="A3" s="378" t="s">
         <v>1099</v>
       </c>
-      <c r="B3" s="377"/>
-      <c r="C3" s="377"/>
-      <c r="D3" s="378"/>
-      <c r="E3" s="377"/>
-      <c r="F3" s="377"/>
-      <c r="G3" s="377"/>
-      <c r="H3" s="377"/>
-      <c r="I3" s="377"/>
-      <c r="J3" s="377"/>
+      <c r="B3" s="378"/>
+      <c r="C3" s="378"/>
+      <c r="D3" s="379"/>
+      <c r="E3" s="378"/>
+      <c r="F3" s="378"/>
+      <c r="G3" s="378"/>
+      <c r="H3" s="378"/>
+      <c r="I3" s="378"/>
+      <c r="J3" s="378"/>
     </row>
     <row r="4" spans="1:38" s="1" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="244" t="s">
@@ -7263,14 +7263,14 @@
       <c r="B4" s="293" t="s">
         <v>14</v>
       </c>
-      <c r="C4" s="380" t="s">
+      <c r="C4" s="381" t="s">
         <v>19</v>
       </c>
-      <c r="D4" s="381"/>
-      <c r="E4" s="379"/>
-      <c r="F4" s="379"/>
-      <c r="G4" s="379"/>
-      <c r="H4" s="379"/>
+      <c r="D4" s="382"/>
+      <c r="E4" s="380"/>
+      <c r="F4" s="380"/>
+      <c r="G4" s="380"/>
+      <c r="H4" s="380"/>
       <c r="I4" s="164" t="s">
         <v>35</v>
       </c>
@@ -8566,10 +8566,10 @@
       <c r="J74" s="284"/>
     </row>
     <row r="75" spans="1:10" s="3" customFormat="1" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A75" s="382" t="s">
+      <c r="A75" s="383" t="s">
         <v>926</v>
       </c>
-      <c r="B75" s="383"/>
+      <c r="B75" s="384"/>
       <c r="C75" s="215"/>
       <c r="D75" s="246"/>
       <c r="E75" s="246"/>
@@ -9668,10 +9668,10 @@
       <c r="M139" s="14"/>
     </row>
     <row r="140" spans="1:13" s="95" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A140" s="376" t="s">
+      <c r="A140" s="377" t="s">
         <v>289</v>
       </c>
-      <c r="B140" s="376"/>
+      <c r="B140" s="377"/>
       <c r="C140" s="189">
         <f>SUM(C8:C139)</f>
         <v>142</v>
@@ -9775,18 +9775,18 @@
       </c>
     </row>
     <row r="2" spans="1:13" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="385" t="s">
+      <c r="A2" s="386" t="s">
         <v>911</v>
       </c>
-      <c r="B2" s="385"/>
-      <c r="C2" s="385"/>
-      <c r="D2" s="385"/>
-      <c r="E2" s="385"/>
-      <c r="F2" s="385"/>
-      <c r="G2" s="385"/>
-      <c r="H2" s="385"/>
-      <c r="I2" s="385"/>
-      <c r="J2" s="385"/>
+      <c r="B2" s="386"/>
+      <c r="C2" s="386"/>
+      <c r="D2" s="386"/>
+      <c r="E2" s="386"/>
+      <c r="F2" s="386"/>
+      <c r="G2" s="386"/>
+      <c r="H2" s="386"/>
+      <c r="I2" s="386"/>
+      <c r="J2" s="386"/>
     </row>
     <row r="3" spans="1:13" s="6" customFormat="1" ht="31.2" x14ac:dyDescent="0.25">
       <c r="A3" s="79" t="s">
@@ -9799,9 +9799,9 @@
         <v>19</v>
       </c>
       <c r="D3" s="106"/>
-      <c r="E3" s="386"/>
-      <c r="F3" s="386"/>
-      <c r="G3" s="386"/>
+      <c r="E3" s="387"/>
+      <c r="F3" s="387"/>
+      <c r="G3" s="387"/>
       <c r="H3" s="79" t="s">
         <v>20</v>
       </c>
@@ -9873,18 +9873,18 @@
       </c>
     </row>
     <row r="6" spans="1:13" ht="24" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="382" t="s">
+      <c r="A6" s="383" t="s">
         <v>747</v>
       </c>
-      <c r="B6" s="383"/>
-      <c r="C6" s="383"/>
-      <c r="D6" s="383"/>
-      <c r="E6" s="383"/>
-      <c r="F6" s="383"/>
-      <c r="G6" s="383"/>
-      <c r="H6" s="383"/>
-      <c r="I6" s="383"/>
-      <c r="J6" s="387"/>
+      <c r="B6" s="384"/>
+      <c r="C6" s="384"/>
+      <c r="D6" s="384"/>
+      <c r="E6" s="384"/>
+      <c r="F6" s="384"/>
+      <c r="G6" s="384"/>
+      <c r="H6" s="384"/>
+      <c r="I6" s="384"/>
+      <c r="J6" s="388"/>
     </row>
     <row r="7" spans="1:13" ht="24" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="247" t="s">
@@ -13613,10 +13613,10 @@
       <c r="J235" s="123"/>
     </row>
     <row r="236" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A236" s="380" t="s">
+      <c r="A236" s="381" t="s">
         <v>289</v>
       </c>
-      <c r="B236" s="384"/>
+      <c r="B236" s="385"/>
       <c r="C236" s="164">
         <f>SUM(C8:C235)</f>
         <v>54</v>
@@ -13736,85 +13736,85 @@
       </c>
     </row>
     <row r="2" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A2" s="388" t="s">
+      <c r="A2" s="389" t="s">
         <v>82</v>
       </c>
-      <c r="B2" s="388"/>
-      <c r="C2" s="388"/>
-      <c r="D2" s="388"/>
-      <c r="E2" s="388"/>
-      <c r="F2" s="388"/>
-      <c r="G2" s="388"/>
-      <c r="H2" s="388"/>
-      <c r="I2" s="388"/>
-      <c r="J2" s="388"/>
-      <c r="K2" s="388"/>
-      <c r="L2" s="388"/>
-      <c r="M2" s="388"/>
-      <c r="N2" s="388"/>
-      <c r="O2" s="388"/>
-      <c r="P2" s="388"/>
-      <c r="Q2" s="388"/>
-      <c r="R2" s="388"/>
-      <c r="S2" s="388"/>
-      <c r="T2" s="388"/>
+      <c r="B2" s="389"/>
+      <c r="C2" s="389"/>
+      <c r="D2" s="389"/>
+      <c r="E2" s="389"/>
+      <c r="F2" s="389"/>
+      <c r="G2" s="389"/>
+      <c r="H2" s="389"/>
+      <c r="I2" s="389"/>
+      <c r="J2" s="389"/>
+      <c r="K2" s="389"/>
+      <c r="L2" s="389"/>
+      <c r="M2" s="389"/>
+      <c r="N2" s="389"/>
+      <c r="O2" s="389"/>
+      <c r="P2" s="389"/>
+      <c r="Q2" s="389"/>
+      <c r="R2" s="389"/>
+      <c r="S2" s="389"/>
+      <c r="T2" s="389"/>
     </row>
     <row r="3" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A3" s="37"/>
       <c r="B3" s="100"/>
-      <c r="R3" s="389"/>
-      <c r="S3" s="390"/>
-      <c r="T3" s="390"/>
+      <c r="R3" s="390"/>
+      <c r="S3" s="391"/>
+      <c r="T3" s="391"/>
     </row>
     <row r="4" spans="1:20" s="101" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="391" t="s">
+      <c r="A4" s="392" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="392" t="s">
+      <c r="B4" s="393" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="393" t="s">
+      <c r="C4" s="394" t="s">
         <v>19</v>
       </c>
-      <c r="D4" s="394"/>
-      <c r="E4" s="391" t="s">
+      <c r="D4" s="395"/>
+      <c r="E4" s="392" t="s">
         <v>33</v>
       </c>
-      <c r="F4" s="391"/>
-      <c r="G4" s="391"/>
-      <c r="H4" s="391"/>
-      <c r="I4" s="391"/>
-      <c r="J4" s="391"/>
-      <c r="K4" s="391"/>
-      <c r="L4" s="391"/>
-      <c r="M4" s="395" t="s">
+      <c r="F4" s="392"/>
+      <c r="G4" s="392"/>
+      <c r="H4" s="392"/>
+      <c r="I4" s="392"/>
+      <c r="J4" s="392"/>
+      <c r="K4" s="392"/>
+      <c r="L4" s="392"/>
+      <c r="M4" s="371" t="s">
         <v>20</v>
       </c>
-      <c r="N4" s="395" t="s">
+      <c r="N4" s="371" t="s">
         <v>34</v>
       </c>
-      <c r="O4" s="397" t="s">
+      <c r="O4" s="396" t="s">
         <v>35</v>
       </c>
-      <c r="P4" s="392" t="s">
+      <c r="P4" s="393" t="s">
         <v>23</v>
       </c>
-      <c r="Q4" s="392" t="s">
+      <c r="Q4" s="393" t="s">
         <v>24</v>
       </c>
-      <c r="R4" s="392" t="s">
+      <c r="R4" s="393" t="s">
         <v>25</v>
       </c>
-      <c r="S4" s="392" t="s">
+      <c r="S4" s="393" t="s">
         <v>26</v>
       </c>
-      <c r="T4" s="399" t="s">
+      <c r="T4" s="398" t="s">
         <v>156</v>
       </c>
     </row>
     <row r="5" spans="1:20" s="101" customFormat="1" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A5" s="391"/>
-      <c r="B5" s="392"/>
+      <c r="A5" s="392"/>
+      <c r="B5" s="393"/>
       <c r="C5" s="250" t="s">
         <v>27</v>
       </c>
@@ -13845,14 +13845,14 @@
       <c r="L5" s="211" t="s">
         <v>30</v>
       </c>
-      <c r="M5" s="396"/>
-      <c r="N5" s="396"/>
-      <c r="O5" s="398"/>
-      <c r="P5" s="392"/>
-      <c r="Q5" s="392"/>
-      <c r="R5" s="392"/>
-      <c r="S5" s="392"/>
-      <c r="T5" s="379"/>
+      <c r="M5" s="372"/>
+      <c r="N5" s="372"/>
+      <c r="O5" s="397"/>
+      <c r="P5" s="393"/>
+      <c r="Q5" s="393"/>
+      <c r="R5" s="393"/>
+      <c r="S5" s="393"/>
+      <c r="T5" s="380"/>
     </row>
     <row r="6" spans="1:20" s="101" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A6" s="211" t="s">
@@ -14510,10 +14510,10 @@
       </c>
     </row>
     <row r="28" spans="1:20" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="376" t="s">
+      <c r="A28" s="377" t="s">
         <v>289</v>
       </c>
-      <c r="B28" s="376"/>
+      <c r="B28" s="377"/>
       <c r="C28" s="211">
         <f>SUM(C26:C27)</f>
         <v>60</v>
@@ -14660,72 +14660,72 @@
       </c>
     </row>
     <row r="2" spans="1:20" ht="15.6" x14ac:dyDescent="0.25">
-      <c r="A2" s="400" t="s">
+      <c r="A2" s="399" t="s">
         <v>100</v>
       </c>
-      <c r="B2" s="400"/>
-      <c r="C2" s="400"/>
-      <c r="D2" s="400"/>
-      <c r="E2" s="400"/>
-      <c r="F2" s="400"/>
-      <c r="G2" s="400"/>
-      <c r="H2" s="400"/>
-      <c r="I2" s="400"/>
-      <c r="J2" s="400"/>
-      <c r="K2" s="400"/>
-      <c r="L2" s="400"/>
-      <c r="M2" s="400"/>
-      <c r="N2" s="400"/>
-      <c r="O2" s="400"/>
-      <c r="P2" s="400"/>
-      <c r="Q2" s="400"/>
+      <c r="B2" s="399"/>
+      <c r="C2" s="399"/>
+      <c r="D2" s="399"/>
+      <c r="E2" s="399"/>
+      <c r="F2" s="399"/>
+      <c r="G2" s="399"/>
+      <c r="H2" s="399"/>
+      <c r="I2" s="399"/>
+      <c r="J2" s="399"/>
+      <c r="K2" s="399"/>
+      <c r="L2" s="399"/>
+      <c r="M2" s="399"/>
+      <c r="N2" s="399"/>
+      <c r="O2" s="399"/>
+      <c r="P2" s="399"/>
+      <c r="Q2" s="399"/>
     </row>
     <row r="3" spans="1:20" s="101" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="397" t="s">
+      <c r="A3" s="396" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="399" t="s">
+      <c r="B3" s="398" t="s">
         <v>18</v>
       </c>
-      <c r="C3" s="391" t="s">
+      <c r="C3" s="392" t="s">
         <v>19</v>
       </c>
-      <c r="D3" s="391"/>
-      <c r="E3" s="391" t="s">
+      <c r="D3" s="392"/>
+      <c r="E3" s="392" t="s">
         <v>33</v>
       </c>
-      <c r="F3" s="391"/>
-      <c r="G3" s="391"/>
-      <c r="H3" s="391"/>
-      <c r="I3" s="391"/>
-      <c r="J3" s="399" t="s">
+      <c r="F3" s="392"/>
+      <c r="G3" s="392"/>
+      <c r="H3" s="392"/>
+      <c r="I3" s="392"/>
+      <c r="J3" s="398" t="s">
         <v>20</v>
       </c>
-      <c r="K3" s="399" t="s">
+      <c r="K3" s="398" t="s">
         <v>21</v>
       </c>
-      <c r="L3" s="399" t="s">
+      <c r="L3" s="398" t="s">
         <v>22</v>
       </c>
-      <c r="M3" s="399" t="s">
+      <c r="M3" s="398" t="s">
         <v>23</v>
       </c>
-      <c r="N3" s="399" t="s">
+      <c r="N3" s="398" t="s">
         <v>24</v>
       </c>
-      <c r="O3" s="399" t="s">
+      <c r="O3" s="398" t="s">
         <v>25</v>
       </c>
-      <c r="P3" s="399" t="s">
+      <c r="P3" s="398" t="s">
         <v>26</v>
       </c>
-      <c r="Q3" s="399" t="s">
+      <c r="Q3" s="398" t="s">
         <v>156</v>
       </c>
     </row>
     <row r="4" spans="1:20" s="101" customFormat="1" ht="62.4" x14ac:dyDescent="0.3">
-      <c r="A4" s="398"/>
-      <c r="B4" s="399"/>
+      <c r="A4" s="397"/>
+      <c r="B4" s="398"/>
       <c r="C4" s="276" t="s">
         <v>27</v>
       </c>
@@ -14747,14 +14747,14 @@
       <c r="I4" s="127" t="s">
         <v>30</v>
       </c>
-      <c r="J4" s="399"/>
-      <c r="K4" s="399"/>
-      <c r="L4" s="399"/>
-      <c r="M4" s="399"/>
-      <c r="N4" s="399"/>
-      <c r="O4" s="399"/>
-      <c r="P4" s="399"/>
-      <c r="Q4" s="379"/>
+      <c r="J4" s="398"/>
+      <c r="K4" s="398"/>
+      <c r="L4" s="398"/>
+      <c r="M4" s="398"/>
+      <c r="N4" s="398"/>
+      <c r="O4" s="398"/>
+      <c r="P4" s="398"/>
+      <c r="Q4" s="380"/>
       <c r="T4" s="101" t="s">
         <v>282</v>
       </c>
@@ -16717,74 +16717,74 @@
       </c>
     </row>
     <row r="2" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A2" s="404" t="s">
+      <c r="A2" s="403" t="s">
         <v>587</v>
       </c>
-      <c r="B2" s="404"/>
-      <c r="C2" s="404"/>
-      <c r="D2" s="404"/>
-      <c r="E2" s="404"/>
-      <c r="F2" s="404"/>
-      <c r="G2" s="404"/>
-      <c r="H2" s="404"/>
-      <c r="I2" s="404"/>
-      <c r="J2" s="404"/>
-      <c r="K2" s="404"/>
-      <c r="L2" s="404"/>
-      <c r="M2" s="404"/>
-      <c r="N2" s="404"/>
-      <c r="O2" s="404"/>
-      <c r="P2" s="404"/>
-      <c r="Q2" s="404"/>
-      <c r="R2" s="404"/>
+      <c r="B2" s="403"/>
+      <c r="C2" s="403"/>
+      <c r="D2" s="403"/>
+      <c r="E2" s="403"/>
+      <c r="F2" s="403"/>
+      <c r="G2" s="403"/>
+      <c r="H2" s="403"/>
+      <c r="I2" s="403"/>
+      <c r="J2" s="403"/>
+      <c r="K2" s="403"/>
+      <c r="L2" s="403"/>
+      <c r="M2" s="403"/>
+      <c r="N2" s="403"/>
+      <c r="O2" s="403"/>
+      <c r="P2" s="403"/>
+      <c r="Q2" s="403"/>
+      <c r="R2" s="403"/>
     </row>
     <row r="3" spans="1:18" s="95" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="379" t="s">
+      <c r="A3" s="380" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="399" t="s">
+      <c r="B3" s="398" t="s">
         <v>14</v>
       </c>
-      <c r="C3" s="379" t="s">
+      <c r="C3" s="380" t="s">
         <v>19</v>
       </c>
-      <c r="D3" s="379"/>
-      <c r="E3" s="379" t="s">
+      <c r="D3" s="380"/>
+      <c r="E3" s="380" t="s">
         <v>33</v>
       </c>
-      <c r="F3" s="379"/>
-      <c r="G3" s="379"/>
-      <c r="H3" s="379"/>
-      <c r="I3" s="379"/>
-      <c r="J3" s="379"/>
-      <c r="K3" s="399" t="s">
+      <c r="F3" s="380"/>
+      <c r="G3" s="380"/>
+      <c r="H3" s="380"/>
+      <c r="I3" s="380"/>
+      <c r="J3" s="380"/>
+      <c r="K3" s="398" t="s">
         <v>20</v>
       </c>
-      <c r="L3" s="399" t="s">
+      <c r="L3" s="398" t="s">
         <v>34</v>
       </c>
-      <c r="M3" s="399" t="s">
+      <c r="M3" s="398" t="s">
         <v>586</v>
       </c>
-      <c r="N3" s="399" t="s">
+      <c r="N3" s="398" t="s">
         <v>23</v>
       </c>
-      <c r="O3" s="399" t="s">
+      <c r="O3" s="398" t="s">
         <v>24</v>
       </c>
-      <c r="P3" s="399" t="s">
+      <c r="P3" s="398" t="s">
         <v>25</v>
       </c>
-      <c r="Q3" s="399" t="s">
+      <c r="Q3" s="398" t="s">
         <v>26</v>
       </c>
-      <c r="R3" s="399" t="s">
+      <c r="R3" s="398" t="s">
         <v>156</v>
       </c>
     </row>
     <row r="4" spans="1:18" s="95" customFormat="1" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A4" s="379"/>
-      <c r="B4" s="399"/>
+      <c r="A4" s="380"/>
+      <c r="B4" s="398"/>
       <c r="C4" s="244" t="s">
         <v>27</v>
       </c>
@@ -16809,14 +16809,14 @@
       <c r="J4" s="164" t="s">
         <v>30</v>
       </c>
-      <c r="K4" s="399"/>
-      <c r="L4" s="399"/>
-      <c r="M4" s="379"/>
-      <c r="N4" s="399"/>
-      <c r="O4" s="399"/>
-      <c r="P4" s="399"/>
-      <c r="Q4" s="399"/>
-      <c r="R4" s="379"/>
+      <c r="K4" s="398"/>
+      <c r="L4" s="398"/>
+      <c r="M4" s="380"/>
+      <c r="N4" s="398"/>
+      <c r="O4" s="398"/>
+      <c r="P4" s="398"/>
+      <c r="Q4" s="398"/>
+      <c r="R4" s="380"/>
     </row>
     <row r="5" spans="1:18" s="3" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
@@ -16879,22 +16879,22 @@
         <v>584</v>
       </c>
       <c r="B6" s="60"/>
-      <c r="C6" s="401"/>
-      <c r="D6" s="402"/>
-      <c r="E6" s="402"/>
-      <c r="F6" s="402"/>
-      <c r="G6" s="402"/>
-      <c r="H6" s="402"/>
-      <c r="I6" s="402"/>
-      <c r="J6" s="402"/>
-      <c r="K6" s="402"/>
-      <c r="L6" s="402"/>
-      <c r="M6" s="402"/>
-      <c r="N6" s="402"/>
-      <c r="O6" s="402"/>
-      <c r="P6" s="402"/>
-      <c r="Q6" s="402"/>
-      <c r="R6" s="403"/>
+      <c r="C6" s="400"/>
+      <c r="D6" s="401"/>
+      <c r="E6" s="401"/>
+      <c r="F6" s="401"/>
+      <c r="G6" s="401"/>
+      <c r="H6" s="401"/>
+      <c r="I6" s="401"/>
+      <c r="J6" s="401"/>
+      <c r="K6" s="401"/>
+      <c r="L6" s="401"/>
+      <c r="M6" s="401"/>
+      <c r="N6" s="401"/>
+      <c r="O6" s="401"/>
+      <c r="P6" s="401"/>
+      <c r="Q6" s="401"/>
+      <c r="R6" s="402"/>
     </row>
     <row r="7" spans="1:18" ht="21.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
@@ -22533,24 +22533,24 @@
       </c>
     </row>
     <row r="2" spans="1:16" s="138" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="400" t="s">
+      <c r="A2" s="399" t="s">
         <v>154</v>
       </c>
-      <c r="B2" s="400"/>
-      <c r="C2" s="400"/>
-      <c r="D2" s="400"/>
-      <c r="E2" s="400"/>
-      <c r="F2" s="400"/>
-      <c r="G2" s="400"/>
-      <c r="H2" s="400"/>
-      <c r="I2" s="400"/>
-      <c r="J2" s="400"/>
-      <c r="K2" s="400"/>
-      <c r="L2" s="400"/>
-      <c r="M2" s="400"/>
-      <c r="N2" s="400"/>
-      <c r="O2" s="400"/>
-      <c r="P2" s="400"/>
+      <c r="B2" s="399"/>
+      <c r="C2" s="399"/>
+      <c r="D2" s="399"/>
+      <c r="E2" s="399"/>
+      <c r="F2" s="399"/>
+      <c r="G2" s="399"/>
+      <c r="H2" s="399"/>
+      <c r="I2" s="399"/>
+      <c r="J2" s="399"/>
+      <c r="K2" s="399"/>
+      <c r="L2" s="399"/>
+      <c r="M2" s="399"/>
+      <c r="N2" s="399"/>
+      <c r="O2" s="399"/>
+      <c r="P2" s="399"/>
     </row>
     <row r="3" spans="1:16" s="36" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="107" t="s">
@@ -24481,10 +24481,10 @@
       <c r="A85" s="108">
         <v>31</v>
       </c>
-      <c r="B85" s="408" t="s">
+      <c r="B85" s="407" t="s">
         <v>226</v>
       </c>
-      <c r="C85" s="409"/>
+      <c r="C85" s="408"/>
       <c r="D85" s="51"/>
       <c r="E85" s="51"/>
       <c r="F85" s="51"/>
@@ -25458,10 +25458,10 @@
       <c r="A123" s="1">
         <v>67</v>
       </c>
-      <c r="B123" s="412" t="s">
+      <c r="B123" s="411" t="s">
         <v>257</v>
       </c>
-      <c r="C123" s="413"/>
+      <c r="C123" s="412"/>
       <c r="D123" s="51"/>
       <c r="E123" s="51"/>
       <c r="F123" s="51"/>
@@ -26308,10 +26308,10 @@
       <c r="A160" s="1">
         <v>104</v>
       </c>
-      <c r="B160" s="410" t="s">
+      <c r="B160" s="409" t="s">
         <v>928</v>
       </c>
-      <c r="C160" s="411"/>
+      <c r="C160" s="410"/>
       <c r="D160" s="51"/>
       <c r="E160" s="51"/>
       <c r="F160" s="51"/>
@@ -26484,10 +26484,10 @@
       <c r="A168" s="1">
         <v>112</v>
       </c>
-      <c r="B168" s="414" t="s">
+      <c r="B168" s="413" t="s">
         <v>957</v>
       </c>
-      <c r="C168" s="415"/>
+      <c r="C168" s="414"/>
       <c r="D168" s="52"/>
       <c r="E168" s="51"/>
       <c r="F168" s="51"/>
@@ -26506,10 +26506,10 @@
       <c r="A169" s="282">
         <v>113</v>
       </c>
-      <c r="B169" s="416" t="s">
+      <c r="B169" s="415" t="s">
         <v>960</v>
       </c>
-      <c r="C169" s="417"/>
+      <c r="C169" s="416"/>
       <c r="D169" s="52"/>
       <c r="E169" s="52"/>
       <c r="F169" s="51"/>
@@ -26528,10 +26528,10 @@
       <c r="A170" s="282">
         <v>114</v>
       </c>
-      <c r="B170" s="416" t="s">
+      <c r="B170" s="415" t="s">
         <v>959</v>
       </c>
-      <c r="C170" s="417"/>
+      <c r="C170" s="416"/>
       <c r="D170" s="52"/>
       <c r="E170" s="52"/>
       <c r="F170" s="51"/>
@@ -26547,11 +26547,11 @@
       <c r="P170" s="56"/>
     </row>
     <row r="171" spans="1:16" s="36" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A171" s="405" t="s">
+      <c r="A171" s="404" t="s">
         <v>596</v>
       </c>
-      <c r="B171" s="406"/>
-      <c r="C171" s="407"/>
+      <c r="B171" s="405"/>
+      <c r="C171" s="406"/>
       <c r="D171" s="217">
         <f>SUBTOTAL(9,D72:D131)</f>
         <v>103</v>
@@ -26656,79 +26656,79 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2927" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="R1" s="420" t="s">
+      <c r="R1" s="419" t="s">
         <v>655</v>
       </c>
-      <c r="S1" s="420"/>
-      <c r="T1" s="420"/>
+      <c r="S1" s="419"/>
+      <c r="T1" s="419"/>
     </row>
     <row r="2" spans="1:2927" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="385" t="s">
+      <c r="A2" s="386" t="s">
         <v>660</v>
       </c>
-      <c r="B2" s="385"/>
-      <c r="C2" s="385"/>
-      <c r="D2" s="385"/>
-      <c r="E2" s="385"/>
-      <c r="F2" s="385"/>
-      <c r="G2" s="385"/>
-      <c r="H2" s="385"/>
-      <c r="I2" s="385"/>
-      <c r="J2" s="385"/>
-      <c r="K2" s="385"/>
-      <c r="L2" s="385"/>
-      <c r="M2" s="385"/>
-      <c r="N2" s="385"/>
-      <c r="O2" s="385"/>
-      <c r="P2" s="385"/>
-      <c r="Q2" s="385"/>
-      <c r="R2" s="385"/>
-      <c r="S2" s="385"/>
-      <c r="T2" s="385"/>
+      <c r="B2" s="386"/>
+      <c r="C2" s="386"/>
+      <c r="D2" s="386"/>
+      <c r="E2" s="386"/>
+      <c r="F2" s="386"/>
+      <c r="G2" s="386"/>
+      <c r="H2" s="386"/>
+      <c r="I2" s="386"/>
+      <c r="J2" s="386"/>
+      <c r="K2" s="386"/>
+      <c r="L2" s="386"/>
+      <c r="M2" s="386"/>
+      <c r="N2" s="386"/>
+      <c r="O2" s="386"/>
+      <c r="P2" s="386"/>
+      <c r="Q2" s="386"/>
+      <c r="R2" s="386"/>
+      <c r="S2" s="386"/>
+      <c r="T2" s="386"/>
     </row>
     <row r="3" spans="1:2927" s="1" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="399" t="s">
+      <c r="A3" s="398" t="s">
         <v>291</v>
       </c>
-      <c r="B3" s="421" t="s">
+      <c r="B3" s="420" t="s">
         <v>14</v>
       </c>
-      <c r="C3" s="379" t="s">
+      <c r="C3" s="380" t="s">
         <v>19</v>
       </c>
-      <c r="D3" s="379"/>
-      <c r="E3" s="379" t="s">
+      <c r="D3" s="380"/>
+      <c r="E3" s="380" t="s">
         <v>33</v>
       </c>
-      <c r="F3" s="379"/>
-      <c r="G3" s="379"/>
-      <c r="H3" s="379"/>
-      <c r="I3" s="379"/>
-      <c r="J3" s="379"/>
-      <c r="K3" s="379"/>
-      <c r="L3" s="379"/>
-      <c r="M3" s="422" t="s">
+      <c r="F3" s="380"/>
+      <c r="G3" s="380"/>
+      <c r="H3" s="380"/>
+      <c r="I3" s="380"/>
+      <c r="J3" s="380"/>
+      <c r="K3" s="380"/>
+      <c r="L3" s="380"/>
+      <c r="M3" s="421" t="s">
         <v>20</v>
       </c>
-      <c r="N3" s="422" t="s">
+      <c r="N3" s="421" t="s">
         <v>292</v>
       </c>
-      <c r="O3" s="379" t="s">
+      <c r="O3" s="380" t="s">
         <v>35</v>
       </c>
-      <c r="P3" s="424" t="s">
+      <c r="P3" s="423" t="s">
         <v>23</v>
       </c>
-      <c r="Q3" s="424" t="s">
+      <c r="Q3" s="423" t="s">
         <v>24</v>
       </c>
-      <c r="R3" s="424" t="s">
+      <c r="R3" s="423" t="s">
         <v>25</v>
       </c>
-      <c r="S3" s="424" t="s">
+      <c r="S3" s="423" t="s">
         <v>26</v>
       </c>
-      <c r="T3" s="399" t="s">
+      <c r="T3" s="398" t="s">
         <v>961</v>
       </c>
       <c r="U3" s="6"/>
@@ -29640,8 +29640,8 @@
       <c r="DHO3" s="6"/>
     </row>
     <row r="4" spans="1:2927" s="1" customFormat="1" ht="31.2" x14ac:dyDescent="0.25">
-      <c r="A4" s="399"/>
-      <c r="B4" s="421"/>
+      <c r="A4" s="398"/>
+      <c r="B4" s="420"/>
       <c r="C4" s="244" t="s">
         <v>27</v>
       </c>
@@ -29672,14 +29672,14 @@
       <c r="L4" s="89" t="s">
         <v>30</v>
       </c>
-      <c r="M4" s="423"/>
-      <c r="N4" s="423"/>
-      <c r="O4" s="379"/>
-      <c r="P4" s="424"/>
-      <c r="Q4" s="424"/>
-      <c r="R4" s="424"/>
-      <c r="S4" s="424"/>
-      <c r="T4" s="379"/>
+      <c r="M4" s="422"/>
+      <c r="N4" s="422"/>
+      <c r="O4" s="380"/>
+      <c r="P4" s="423"/>
+      <c r="Q4" s="423"/>
+      <c r="R4" s="423"/>
+      <c r="S4" s="423"/>
+      <c r="T4" s="380"/>
       <c r="U4" s="6"/>
       <c r="V4" s="6"/>
       <c r="W4" s="6"/>
@@ -35558,12 +35558,12 @@
       <c r="DHO5" s="6"/>
     </row>
     <row r="6" spans="1:2927" s="3" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="418" t="s">
+      <c r="A6" s="417" t="s">
         <v>627</v>
       </c>
-      <c r="B6" s="419"/>
-      <c r="C6" s="419"/>
-      <c r="D6" s="419"/>
+      <c r="B6" s="418"/>
+      <c r="C6" s="418"/>
+      <c r="D6" s="418"/>
       <c r="E6" s="205"/>
       <c r="F6" s="205"/>
       <c r="G6" s="205"/>
@@ -68365,10 +68365,10 @@
       <c r="T37" s="108"/>
     </row>
     <row r="38" spans="1:20" s="101" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="376" t="s">
+      <c r="A38" s="377" t="s">
         <v>289</v>
       </c>
-      <c r="B38" s="376"/>
+      <c r="B38" s="377"/>
       <c r="C38" s="164"/>
       <c r="D38" s="164"/>
       <c r="E38" s="164"/>
@@ -68473,48 +68473,48 @@
       <c r="J2" s="222"/>
     </row>
     <row r="3" spans="1:10" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="360" t="s">
+      <c r="A3" s="432" t="s">
         <v>939</v>
       </c>
-      <c r="B3" s="360"/>
-      <c r="C3" s="360"/>
-      <c r="D3" s="360"/>
-      <c r="E3" s="360"/>
-      <c r="F3" s="360"/>
-      <c r="G3" s="360"/>
-      <c r="H3" s="360"/>
-      <c r="I3" s="360"/>
-      <c r="J3" s="360"/>
+      <c r="B3" s="432"/>
+      <c r="C3" s="432"/>
+      <c r="D3" s="432"/>
+      <c r="E3" s="432"/>
+      <c r="F3" s="432"/>
+      <c r="G3" s="432"/>
+      <c r="H3" s="432"/>
+      <c r="I3" s="432"/>
+      <c r="J3" s="432"/>
     </row>
     <row r="4" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A4" s="361" t="s">
+      <c r="A4" s="429" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="361" t="s">
+      <c r="B4" s="429" t="s">
         <v>14</v>
       </c>
-      <c r="C4" s="362" t="s">
+      <c r="C4" s="433" t="s">
         <v>19</v>
       </c>
-      <c r="D4" s="362"/>
-      <c r="E4" s="362" t="s">
+      <c r="D4" s="433"/>
+      <c r="E4" s="433" t="s">
         <v>940</v>
       </c>
-      <c r="F4" s="362"/>
-      <c r="G4" s="362"/>
-      <c r="H4" s="361" t="s">
+      <c r="F4" s="433"/>
+      <c r="G4" s="433"/>
+      <c r="H4" s="429" t="s">
         <v>941</v>
       </c>
-      <c r="I4" s="363" t="s">
+      <c r="I4" s="434" t="s">
         <v>942</v>
       </c>
-      <c r="J4" s="364" t="s">
+      <c r="J4" s="435" t="s">
         <v>962</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="361"/>
-      <c r="B5" s="361"/>
+      <c r="A5" s="429"/>
+      <c r="B5" s="429"/>
       <c r="C5" s="227" t="s">
         <v>27</v>
       </c>
@@ -68530,15 +68530,15 @@
       <c r="G5" s="226" t="s">
         <v>35</v>
       </c>
-      <c r="H5" s="361"/>
-      <c r="I5" s="363"/>
-      <c r="J5" s="364"/>
+      <c r="H5" s="429"/>
+      <c r="I5" s="434"/>
+      <c r="J5" s="435"/>
     </row>
     <row r="6" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A6" s="366" t="s">
+      <c r="A6" s="425" t="s">
         <v>1049</v>
       </c>
-      <c r="B6" s="367"/>
+      <c r="B6" s="426"/>
       <c r="C6" s="227"/>
       <c r="D6" s="227"/>
       <c r="E6" s="226"/>
@@ -69959,10 +69959,10 @@
       <c r="J93" s="328"/>
     </row>
     <row r="94" spans="1:10" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A94" s="361" t="s">
+      <c r="A94" s="429" t="s">
         <v>1047</v>
       </c>
-      <c r="B94" s="361"/>
+      <c r="B94" s="429"/>
       <c r="C94" s="229"/>
       <c r="D94" s="229"/>
       <c r="E94" s="229"/>
@@ -69989,10 +69989,10 @@
       <c r="J95" s="229"/>
     </row>
     <row r="96" spans="1:10" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A96" s="370" t="s">
+      <c r="A96" s="430" t="s">
         <v>596</v>
       </c>
-      <c r="B96" s="371"/>
+      <c r="B96" s="431"/>
       <c r="C96" s="304"/>
       <c r="D96" s="304"/>
       <c r="E96" s="304"/>
@@ -70003,18 +70003,18 @@
       <c r="J96" s="304"/>
     </row>
     <row r="97" spans="1:10" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A97" s="365" t="s">
+      <c r="A97" s="424" t="s">
         <v>1050</v>
       </c>
-      <c r="B97" s="365"/>
-      <c r="C97" s="365"/>
-      <c r="D97" s="365"/>
-      <c r="E97" s="365"/>
-      <c r="F97" s="365"/>
-      <c r="G97" s="365"/>
-      <c r="H97" s="365"/>
-      <c r="I97" s="365"/>
-      <c r="J97" s="365"/>
+      <c r="B97" s="424"/>
+      <c r="C97" s="424"/>
+      <c r="D97" s="424"/>
+      <c r="E97" s="424"/>
+      <c r="F97" s="424"/>
+      <c r="G97" s="424"/>
+      <c r="H97" s="424"/>
+      <c r="I97" s="424"/>
+      <c r="J97" s="424"/>
     </row>
     <row r="98" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A98" s="327">
@@ -70423,10 +70423,10 @@
       <c r="J122" s="229"/>
     </row>
     <row r="123" spans="1:10" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A123" s="368" t="s">
+      <c r="A123" s="427" t="s">
         <v>596</v>
       </c>
-      <c r="B123" s="369"/>
+      <c r="B123" s="428"/>
       <c r="C123" s="229"/>
       <c r="D123" s="229"/>
       <c r="E123" s="229"/>
@@ -70445,11 +70445,6 @@
     </filterColumn>
   </autoFilter>
   <mergeCells count="13">
-    <mergeCell ref="A97:J97"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="A123:B123"/>
-    <mergeCell ref="A94:B94"/>
-    <mergeCell ref="A96:B96"/>
     <mergeCell ref="A3:J3"/>
     <mergeCell ref="A4:A5"/>
     <mergeCell ref="B4:B5"/>
@@ -70458,6 +70453,11 @@
     <mergeCell ref="H4:H5"/>
     <mergeCell ref="I4:I5"/>
     <mergeCell ref="J4:J5"/>
+    <mergeCell ref="A97:J97"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="A123:B123"/>
+    <mergeCell ref="A94:B94"/>
+    <mergeCell ref="A96:B96"/>
   </mergeCells>
   <conditionalFormatting sqref="D1">
     <cfRule type="iconSet" priority="2">

</xml_diff>